<commit_message>
Muutettu väärin oleva pyöristys
</commit_message>
<xml_diff>
--- a/Aktiviteetit/Vuosi_2025/Aktiviteetit_Heinäkuu.xlsx
+++ b/Aktiviteetit/Vuosi_2025/Aktiviteetit_Heinäkuu.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,14 +473,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Morning Run</t>
+          <t>Afternoon Run</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9.31</v>
+        <v>26.26</v>
       </c>
       <c r="C2" t="n">
-        <v>3983</v>
+        <v>9410</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -489,32 +489,32 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2025-07-14T09:56:26Z</t>
+          <t>2025-07-28T13:02:00Z</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>07:08</t>
+          <t>05:58</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>2.339</v>
+        <v>2.791</v>
       </c>
       <c r="H2" t="n">
-        <v>140.5</v>
+        <v>141.3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Afternoon Run</t>
+          <t>Lunch Run</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18.41</v>
+        <v>10.2</v>
       </c>
       <c r="C3" t="n">
-        <v>5523</v>
+        <v>3667</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -523,32 +523,32 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025-07-12T16:48:18Z</t>
+          <t>2025-07-27T11:20:36Z</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>05:00</t>
+          <t>05:60</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>3.334</v>
+        <v>2.781</v>
       </c>
       <c r="H3" t="n">
-        <v>168.3</v>
+        <v>137.9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Intervallit</t>
+          <t>Afternoon Run</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11.05</v>
+        <v>6.21</v>
       </c>
       <c r="C4" t="n">
-        <v>3267</v>
+        <v>2253</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -557,19 +557,19 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2025-07-10T11:46:41Z</t>
+          <t>2025-07-26T14:32:20Z</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>04:56</t>
+          <t>06:03</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>3.383</v>
+        <v>2.757</v>
       </c>
       <c r="H4" t="n">
-        <v>158.5</v>
+        <v>136.5</v>
       </c>
     </row>
     <row r="5">
@@ -579,10 +579,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12</v>
+        <v>13.13</v>
       </c>
       <c r="C5" t="n">
-        <v>4688</v>
+        <v>4996</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -591,32 +591,32 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2025-07-09T12:24:49Z</t>
+          <t>2025-07-24T11:35:34Z</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>06:31</t>
+          <t>06:21</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>2.561</v>
+        <v>2.627</v>
       </c>
       <c r="H5" t="n">
-        <v>139.5</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Säbä</t>
+          <t>Morning Run</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6.41</v>
+        <v>10.34</v>
       </c>
       <c r="C6" t="n">
-        <v>5900</v>
+        <v>3707</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -625,32 +625,32 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2025-07-08T19:33:57Z</t>
+          <t>2025-07-23T10:22:52Z</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>05:59</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1.086</v>
+        <v>2.79</v>
       </c>
       <c r="H6" t="n">
-        <v>131.2</v>
+        <v>138.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Night Run</t>
+          <t>Intervallit</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9.09</v>
+        <v>11</v>
       </c>
       <c r="C7" t="n">
-        <v>3666</v>
+        <v>3457</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -659,32 +659,32 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2025-07-07T21:57:25Z</t>
+          <t>2025-07-22T19:25:58Z</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>06:43</t>
+          <t>05:14</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>2.479</v>
+        <v>3.181</v>
       </c>
       <c r="H7" t="n">
-        <v>138.6</v>
+        <v>149.8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Afternoon Run</t>
+          <t>Lunch Run</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>21.27</v>
+        <v>10.31</v>
       </c>
       <c r="C8" t="n">
-        <v>7807</v>
+        <v>4098</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -693,32 +693,32 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2025-07-05T16:17:54Z</t>
+          <t>2025-07-21T11:27:46Z</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>06:07</t>
+          <t>06:37</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>2.724</v>
+        <v>2.517</v>
       </c>
       <c r="H8" t="n">
-        <v>145.7</v>
+        <v>140.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Vetoja</t>
+          <t>Evening Run</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7.06</v>
+        <v>22.43</v>
       </c>
       <c r="C9" t="n">
-        <v>2404</v>
+        <v>7971</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -727,32 +727,32 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2025-07-03T20:37:43Z</t>
+          <t>2025-07-19T20:00:40Z</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>05:41</t>
+          <t>05:55</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2.938</v>
+        <v>2.814</v>
       </c>
       <c r="H9" t="n">
-        <v>153.8</v>
+        <v>148.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Morning Run</t>
+          <t>Evening Run</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>10.65</v>
+        <v>10.15</v>
       </c>
       <c r="C10" t="n">
-        <v>4308</v>
+        <v>3886</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -761,32 +761,32 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2025-07-02T10:27:49Z</t>
+          <t>2025-07-18T18:01:02Z</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>06:45</t>
+          <t>06:23</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2.471</v>
+        <v>2.612</v>
       </c>
       <c r="H10" t="n">
-        <v>135</v>
+        <v>136.8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Säbä</t>
+          <t>Intervallit</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5.03</v>
+        <v>10.21</v>
       </c>
       <c r="C11" t="n">
-        <v>4714</v>
+        <v>3010</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -795,52 +795,426 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2025-07-01T20:42:49Z</t>
+          <t>2025-07-17T12:39:36Z</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>15:37</t>
+          <t>04:55</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>1.067</v>
+        <v>3.393</v>
       </c>
       <c r="H11" t="n">
-        <v>142.1</v>
+        <v>158</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Afternoon Run</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="C12" t="n">
+        <v>5642</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2025-07-15T13:21:14Z</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>06:40</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>2.498</v>
+      </c>
+      <c r="H12" t="n">
+        <v>142.1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Morning Run</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>9.31</v>
+      </c>
+      <c r="C13" t="n">
+        <v>3983</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2025-07-14T09:56:26Z</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>07:08</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>2.339</v>
+      </c>
+      <c r="H13" t="n">
+        <v>140.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Afternoon Run</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>18.41</v>
+      </c>
+      <c r="C14" t="n">
+        <v>5523</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2025-07-12T16:48:18Z</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>3.334</v>
+      </c>
+      <c r="H14" t="n">
+        <v>168.3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Intervallit</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>11.05</v>
+      </c>
+      <c r="C15" t="n">
+        <v>3267</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2025-07-10T11:46:41Z</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>04:56</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>3.383</v>
+      </c>
+      <c r="H15" t="n">
+        <v>158.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Lunch Run</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>12</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4688</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2025-07-09T12:24:49Z</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>06:31</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>2.561</v>
+      </c>
+      <c r="H16" t="n">
+        <v>139.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Säbä</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="C17" t="n">
+        <v>5900</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2025-07-08T19:33:57Z</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1.086</v>
+      </c>
+      <c r="H17" t="n">
+        <v>131.2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Night Run</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>9.09</v>
+      </c>
+      <c r="C18" t="n">
+        <v>3666</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2025-07-07T21:57:25Z</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>06:43</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>2.479</v>
+      </c>
+      <c r="H18" t="n">
+        <v>138.6</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Afternoon Run</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>21.27</v>
+      </c>
+      <c r="C19" t="n">
+        <v>7807</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2025-07-05T16:17:54Z</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>06:07</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>2.724</v>
+      </c>
+      <c r="H19" t="n">
+        <v>145.7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Vetoja</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>7.06</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2404</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2025-07-03T20:37:43Z</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>05:41</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>2.938</v>
+      </c>
+      <c r="H20" t="n">
+        <v>153.8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Morning Run</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4308</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2025-07-02T10:27:49Z</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>06:45</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>2.471</v>
+      </c>
+      <c r="H21" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Säbä</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="C22" t="n">
+        <v>4714</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2025-07-01T20:42:49Z</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>15:37</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>1.067</v>
+      </c>
+      <c r="H22" t="n">
+        <v>142.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>Alkulämpöfutis</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B23" t="n">
         <v>1.4</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C23" t="n">
         <v>760</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>2025-07-01T20:24:46Z</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>09:03</t>
         </is>
       </c>
-      <c r="G12" t="n">
+      <c r="G23" t="n">
         <v>1.839</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H23" t="n">
         <v>135.1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Huomattu Bugi, jossa jostain syystä olin katsonu aktiviteetit ennen vikaa päivää enkä ennen seuraavan kuukauden ekaa päivää. Tämä korjattu toivottavasti nyt ei tule bugeja enään. Tämän takia testit olisi hyvä
</commit_message>
<xml_diff>
--- a/Aktiviteetit/Vuosi_2025/Aktiviteetit_Heinäkuu.xlsx
+++ b/Aktiviteetit/Vuosi_2025/Aktiviteetit_Heinäkuu.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,14 +473,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Afternoon Run</t>
+          <t>Tempo 10K</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>26.26</v>
+        <v>10.03</v>
       </c>
       <c r="C2" t="n">
-        <v>9410</v>
+        <v>2600</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -489,19 +489,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2025-07-28T13:02:00Z</t>
+          <t>2025-07-31T18:50:22Z</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>05:58</t>
+          <t>04:19</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>2.791</v>
+        <v>3.859</v>
       </c>
       <c r="H2" t="n">
-        <v>141.3</v>
+        <v>169.5</v>
       </c>
     </row>
     <row r="3">
@@ -511,10 +511,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10.2</v>
+        <v>12.13</v>
       </c>
       <c r="C3" t="n">
-        <v>3667</v>
+        <v>4427</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -523,19 +523,19 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025-07-27T11:20:36Z</t>
+          <t>2025-07-30T11:47:49Z</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>05:60</t>
+          <t>06:04</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>2.781</v>
+        <v>2.741</v>
       </c>
       <c r="H3" t="n">
-        <v>137.9</v>
+        <v>142.2</v>
       </c>
     </row>
     <row r="4">
@@ -545,10 +545,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6.21</v>
+        <v>26.26</v>
       </c>
       <c r="C4" t="n">
-        <v>2253</v>
+        <v>9410</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -557,19 +557,19 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2025-07-26T14:32:20Z</t>
+          <t>2025-07-28T13:02:00Z</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>06:03</t>
+          <t>05:58</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>2.757</v>
+        <v>2.791</v>
       </c>
       <c r="H4" t="n">
-        <v>136.5</v>
+        <v>141.3</v>
       </c>
     </row>
     <row r="5">
@@ -579,10 +579,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>13.13</v>
+        <v>10.2</v>
       </c>
       <c r="C5" t="n">
-        <v>4996</v>
+        <v>3667</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -591,32 +591,32 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2025-07-24T11:35:34Z</t>
+          <t>2025-07-27T11:20:36Z</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>05:59</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>2.627</v>
+        <v>2.781</v>
       </c>
       <c r="H5" t="n">
-        <v>141</v>
+        <v>137.9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Morning Run</t>
+          <t>Afternoon Run</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10.34</v>
+        <v>6.21</v>
       </c>
       <c r="C6" t="n">
-        <v>3707</v>
+        <v>2253</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -625,32 +625,32 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2025-07-23T10:22:52Z</t>
+          <t>2025-07-26T14:32:20Z</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>05:59</t>
+          <t>06:02</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>2.79</v>
+        <v>2.757</v>
       </c>
       <c r="H6" t="n">
-        <v>138.6</v>
+        <v>136.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Intervallit</t>
+          <t>Lunch Run</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>11</v>
+        <v>13.13</v>
       </c>
       <c r="C7" t="n">
-        <v>3457</v>
+        <v>4996</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -659,32 +659,32 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2025-07-22T19:25:58Z</t>
+          <t>2025-07-24T11:35:34Z</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>05:14</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>3.181</v>
+        <v>2.627</v>
       </c>
       <c r="H7" t="n">
-        <v>149.8</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Lunch Run</t>
+          <t>Morning Run</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10.31</v>
+        <v>10.34</v>
       </c>
       <c r="C8" t="n">
-        <v>4098</v>
+        <v>3707</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -693,32 +693,32 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2025-07-21T11:27:46Z</t>
+          <t>2025-07-23T10:22:52Z</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>06:37</t>
+          <t>05:58</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>2.517</v>
+        <v>2.79</v>
       </c>
       <c r="H8" t="n">
-        <v>140.7</v>
+        <v>138.6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Evening Run</t>
+          <t>Intervallit</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>22.43</v>
+        <v>11</v>
       </c>
       <c r="C9" t="n">
-        <v>7971</v>
+        <v>3457</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -727,32 +727,32 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2025-07-19T20:00:40Z</t>
+          <t>2025-07-22T19:25:58Z</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>05:55</t>
+          <t>05:14</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2.814</v>
+        <v>3.181</v>
       </c>
       <c r="H9" t="n">
-        <v>148.1</v>
+        <v>149.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Evening Run</t>
+          <t>Lunch Run</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>10.15</v>
+        <v>10.31</v>
       </c>
       <c r="C10" t="n">
-        <v>3886</v>
+        <v>4098</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -761,32 +761,32 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2025-07-18T18:01:02Z</t>
+          <t>2025-07-21T11:27:46Z</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>06:23</t>
+          <t>06:37</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2.612</v>
+        <v>2.517</v>
       </c>
       <c r="H10" t="n">
-        <v>136.8</v>
+        <v>140.7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Intervallit</t>
+          <t>Evening Run</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>10.21</v>
+        <v>22.43</v>
       </c>
       <c r="C11" t="n">
-        <v>3010</v>
+        <v>7971</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -795,32 +795,32 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2025-07-17T12:39:36Z</t>
+          <t>2025-07-19T20:00:40Z</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>04:55</t>
+          <t>05:55</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>3.393</v>
+        <v>2.814</v>
       </c>
       <c r="H11" t="n">
-        <v>158</v>
+        <v>148.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Afternoon Run</t>
+          <t>Evening Run</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>14.1</v>
+        <v>10.15</v>
       </c>
       <c r="C12" t="n">
-        <v>5642</v>
+        <v>3886</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -829,32 +829,32 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2025-07-15T13:21:14Z</t>
+          <t>2025-07-18T18:01:02Z</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>06:22</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>2.498</v>
+        <v>2.612</v>
       </c>
       <c r="H12" t="n">
-        <v>142.1</v>
+        <v>136.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Morning Run</t>
+          <t>Intervallit</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>9.31</v>
+        <v>10.21</v>
       </c>
       <c r="C13" t="n">
-        <v>3983</v>
+        <v>3010</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -863,19 +863,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2025-07-14T09:56:26Z</t>
+          <t>2025-07-17T12:39:36Z</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>07:08</t>
+          <t>04:54</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2.339</v>
+        <v>3.393</v>
       </c>
       <c r="H13" t="n">
-        <v>140.5</v>
+        <v>158</v>
       </c>
     </row>
     <row r="14">
@@ -885,10 +885,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>18.41</v>
+        <v>14.1</v>
       </c>
       <c r="C14" t="n">
-        <v>5523</v>
+        <v>5642</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -897,32 +897,32 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025-07-12T16:48:18Z</t>
+          <t>2025-07-15T13:21:14Z</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>05:00</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>3.334</v>
+        <v>2.498</v>
       </c>
       <c r="H14" t="n">
-        <v>168.3</v>
+        <v>142.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Intervallit</t>
+          <t>Morning Run</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>11.05</v>
+        <v>9.31</v>
       </c>
       <c r="C15" t="n">
-        <v>3267</v>
+        <v>3983</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -931,32 +931,32 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2025-07-10T11:46:41Z</t>
+          <t>2025-07-14T09:56:26Z</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>04:56</t>
+          <t>07:07</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>3.383</v>
+        <v>2.339</v>
       </c>
       <c r="H15" t="n">
-        <v>158.5</v>
+        <v>140.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Lunch Run</t>
+          <t>Afternoon Run</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>12</v>
+        <v>18.41</v>
       </c>
       <c r="C16" t="n">
-        <v>4688</v>
+        <v>5523</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -965,32 +965,32 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2025-07-09T12:24:49Z</t>
+          <t>2025-07-12T16:48:18Z</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>06:31</t>
+          <t>05:00</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>2.561</v>
+        <v>3.334</v>
       </c>
       <c r="H16" t="n">
-        <v>139.5</v>
+        <v>168.3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Säbä</t>
+          <t>Intervallit</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>6.41</v>
+        <v>11.05</v>
       </c>
       <c r="C17" t="n">
-        <v>5900</v>
+        <v>3267</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -999,32 +999,32 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2025-07-08T19:33:57Z</t>
+          <t>2025-07-10T11:46:41Z</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>04:55</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>1.086</v>
+        <v>3.383</v>
       </c>
       <c r="H17" t="n">
-        <v>131.2</v>
+        <v>158.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Night Run</t>
+          <t>Lunch Run</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>9.09</v>
+        <v>12</v>
       </c>
       <c r="C18" t="n">
-        <v>3666</v>
+        <v>4688</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1033,32 +1033,32 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2025-07-07T21:57:25Z</t>
+          <t>2025-07-09T12:24:49Z</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>06:43</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>2.479</v>
+        <v>2.561</v>
       </c>
       <c r="H18" t="n">
-        <v>138.6</v>
+        <v>139.5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Afternoon Run</t>
+          <t>Säbä</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>21.27</v>
+        <v>6.41</v>
       </c>
       <c r="C19" t="n">
-        <v>7807</v>
+        <v>5900</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1067,32 +1067,32 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2025-07-05T16:17:54Z</t>
+          <t>2025-07-08T19:33:57Z</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>06:07</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>2.724</v>
+        <v>1.086</v>
       </c>
       <c r="H19" t="n">
-        <v>145.7</v>
+        <v>131.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Vetoja</t>
+          <t>Night Run</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>7.06</v>
+        <v>9.09</v>
       </c>
       <c r="C20" t="n">
-        <v>2404</v>
+        <v>3666</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1101,32 +1101,32 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2025-07-03T20:37:43Z</t>
+          <t>2025-07-07T21:57:25Z</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>05:41</t>
+          <t>06:43</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>2.938</v>
+        <v>2.479</v>
       </c>
       <c r="H20" t="n">
-        <v>153.8</v>
+        <v>138.6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Morning Run</t>
+          <t>Afternoon Run</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>10.65</v>
+        <v>21.27</v>
       </c>
       <c r="C21" t="n">
-        <v>4308</v>
+        <v>7807</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1135,32 +1135,32 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2025-07-02T10:27:49Z</t>
+          <t>2025-07-05T16:17:54Z</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>06:45</t>
+          <t>06:07</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>2.471</v>
+        <v>2.724</v>
       </c>
       <c r="H21" t="n">
-        <v>135</v>
+        <v>145.7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Säbä</t>
+          <t>Vetoja</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>5.03</v>
+        <v>7.06</v>
       </c>
       <c r="C22" t="n">
-        <v>4714</v>
+        <v>2404</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1169,52 +1169,120 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2025-07-01T20:42:49Z</t>
+          <t>2025-07-03T20:37:43Z</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>15:37</t>
+          <t>05:40</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>1.067</v>
+        <v>2.938</v>
       </c>
       <c r="H22" t="n">
-        <v>142.1</v>
+        <v>153.8</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>Morning Run</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="C23" t="n">
+        <v>4308</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2025-07-02T10:27:49Z</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>06:44</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>2.471</v>
+      </c>
+      <c r="H23" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Säbä</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="C24" t="n">
+        <v>4714</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2025-07-01T20:42:49Z</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>15:37</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>1.067</v>
+      </c>
+      <c r="H24" t="n">
+        <v>142.1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>Alkulämpöfutis</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B25" t="n">
         <v>1.4</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C25" t="n">
         <v>760</v>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>2025-07-01T20:24:46Z</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>09:03</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
         <v>1.839</v>
       </c>
-      <c r="H23" t="n">
+      <c r="H25" t="n">
         <v>135.1</v>
       </c>
     </row>

</xml_diff>